<commit_message>
Corregir mayúsculas en el link de GitHub Pages
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D5QSopUe1AGeXzsxrqVKzM
</commit_message>
<xml_diff>
--- a/plantilla-paquetes.xlsx
+++ b/plantilla-paquetes.xlsx
@@ -2079,9 +2079,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -2124,13 +2122,11 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>App: https://victormenav.github.io/rutafacilcr/</t>
+          <t>App: https://victormenav.github.io/RutafacilCR/</t>
         </is>
       </c>
     </row>

</xml_diff>